<commit_message>
plan: shift book submission to Aug 30, sync task statuses to verified state, fix build-views v2 default
</commit_message>
<xml_diff>
--- a/scripts/ticoprojectplanv2.xlsx
+++ b/scripts/ticoprojectplanv2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Project Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Track Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="H12" s="59" t="inlineStr">
         <is>
-          <t>(Author, Year) מתהפך ל-(Year, Author) body-wide · עטיפת פלט הציטוט ב-\LR דרך biblatex cite-hook (לא \renewcommand — natbib שובר) · test-build + בדיקה: single / et al. / multi-cite · מעל אימות ביבליו׳</t>
+          <t>קוד \textenglish+\mbox ✓ (אומת); נותר רסטור-PDF: single / et al. / multi-cite</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="C15" s="49" t="inlineStr">
         <is>
-          <t>פרק 9 (דיון)</t>
+          <t>✅ פרק 9 (דיון)</t>
         </is>
       </c>
       <c r="D15" s="50" t="n">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="C16" s="59" t="inlineStr">
         <is>
-          <t>Abstract אנגלית + עברית</t>
+          <t>✅ Abstract אנגלית</t>
         </is>
       </c>
       <c r="D16" s="60" t="n">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="H16" s="59" t="inlineStr">
         <is>
-          <t>לפי תקנון HIT</t>
+          <t>אנגלי גמור ומאומת-מקור · תקציר עברי לא נדרש (תקנון §ז, ספר עברי)</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="C17" s="49" t="inlineStr">
         <is>
-          <t>הקפאת תוכן + הגהה + בנייה סופית</t>
+          <t>הקפאת תוכן + הגהה + בנייה סופית + הזמנת דפוס (Zami)</t>
         </is>
       </c>
       <c r="D17" s="50" t="n">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="H45" s="49" t="inlineStr">
         <is>
-          <t>אם הדמו קורס בלילה בריצה לא-מאוישת — זיהוי + הפעלה-מחדש אוטומטית</t>
+          <t>אם הדמו קורס בלילה בריצה לא-מאוישת — זיהוי + הפעלה-מחדש אוטומטית · ⚠ טרם התחיל — אפס artifacts (deploy+אמינות 14 יום); תאריך מיושן</t>
         </is>
       </c>
     </row>
@@ -2407,12 +2407,12 @@
       </c>
       <c r="G56" s="61" t="inlineStr">
         <is>
-          <t>DESIGN</t>
+          <t>DEV</t>
         </is>
       </c>
       <c r="H56" s="59" t="inlineStr">
         <is>
-          <t>פריסת הדפסה/QR; תלוי בפיצ'ר ה-export (משימה 32)</t>
+          <t>פריסת הדפסה/QR; תלוי בפיצ'ר ה-export (משימה 32) · QL-800 label — אפס קוד, מנדטורי, בנייה מאפס</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="H65" s="49" t="inlineStr">
         <is>
-          <t>תוכן סופי לפני בנייה+הדפסה</t>
+          <t>תוכן סופי לפני בנייה+הדפסה · גזור ל-lead-time של Zami — אמת השבוע</t>
         </is>
       </c>
     </row>
@@ -2719,10 +2719,10 @@
         </is>
       </c>
       <c r="D67" s="50" t="n">
-        <v>46238</v>
+        <v>46264</v>
       </c>
       <c r="E67" s="50" t="n">
-        <v>46238</v>
+        <v>46264</v>
       </c>
       <c r="F67" s="47">
         <f>E63-D63+1</f>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="H67" s="49" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>דיגיטלי · 30.8 רשת ביטחון; יעד אמיתי = מודפס לפתיחה 6.8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
plan: add 2-week video + live-station bars
</commit_message>
<xml_diff>
--- a/scripts/ticoprojectplanv2.xlsx
+++ b/scripts/ticoprojectplanv2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Project Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Track Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="0&quot; days&quot;"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -756,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="39" min="1" max="1"/>
@@ -781,6 +782,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="40">
       <c r="A4" s="43" t="inlineStr">
         <is>
@@ -1723,204 +1725,202 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="40">
-      <c r="A35" s="47" t="n">
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>26b</t>
+        </is>
+      </c>
+      <c r="B35" s="58" t="inlineStr">
+        <is>
+          <t>אפליקציה</t>
+        </is>
+      </c>
+      <c r="C35" s="59" t="inlineStr">
+        <is>
+          <t>portrait reflow (display-&gt;portrait)</t>
+        </is>
+      </c>
+      <c r="D35" s="60" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E35" s="60" t="n">
+        <v>46211</v>
+      </c>
+      <c r="F35" s="57" t="n"/>
+      <c r="G35" s="61" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+      <c r="H35" s="59" t="inlineStr">
+        <is>
+          <t>חוסם onboarding+peek - קודם לכל UI של התחנה</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="40">
+      <c r="A36" s="47" t="n">
         <v>27</v>
       </c>
-      <c r="B35" s="48" t="inlineStr">
+      <c r="B36" s="48" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C35" s="49" t="inlineStr">
+      <c r="C36" s="49" t="inlineStr">
         <is>
           <t>חיבור tico-orb ל-TTS envelope + VAD</t>
         </is>
       </c>
-      <c r="D35" s="50" t="n">
+      <c r="D36" s="50" t="n">
         <v>46181</v>
       </c>
-      <c r="E35" s="50" t="n">
+      <c r="E36" s="50" t="n">
         <v>46191</v>
       </c>
-      <c r="F35" s="47">
+      <c r="F36" s="47">
         <f>E34-D34+1</f>
         <v/>
       </c>
-      <c r="G35" s="51" t="inlineStr">
+      <c r="G36" s="51" t="inlineStr">
         <is>
           <t>DEV</t>
         </is>
       </c>
-      <c r="H35" s="49" t="inlineStr">
+      <c r="H36" s="49" t="inlineStr">
         <is>
           <t>פה לפי אמפליטודה; מעברי-מצב</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="40">
-      <c r="A36" s="57" t="n">
+    <row r="37" ht="15" customHeight="1" s="40">
+      <c r="A37" s="57" t="n">
         <v>28</v>
       </c>
-      <c r="B36" s="58" t="inlineStr">
+      <c r="B37" s="58" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C36" s="59" t="inlineStr">
+      <c r="C37" s="59" t="inlineStr">
         <is>
           <t>AGT-06 אימות מקצה-לקצה</t>
         </is>
       </c>
-      <c r="D36" s="60" t="n">
+      <c r="D37" s="60" t="n">
         <v>46183</v>
       </c>
-      <c r="E36" s="60" t="n">
+      <c r="E37" s="60" t="n">
         <v>46189</v>
       </c>
-      <c r="F36" s="57">
+      <c r="F37" s="57">
         <f>E35-D35+1</f>
         <v/>
       </c>
-      <c r="G36" s="61" t="inlineStr">
+      <c r="G37" s="61" t="inlineStr">
         <is>
           <t>DEV</t>
         </is>
       </c>
-      <c r="H36" s="59" t="inlineStr">
+      <c r="H37" s="59" t="inlineStr">
         <is>
           <t>frontend לא אומת בזרימה מלאה</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="40">
-      <c r="A37" s="47" t="n">
+    <row r="38" ht="15" customHeight="1" s="40">
+      <c r="A38" s="47" t="n">
         <v>29</v>
       </c>
-      <c r="B37" s="48" t="inlineStr">
+      <c r="B38" s="48" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C37" s="49" t="inlineStr">
+      <c r="C38" s="49" t="inlineStr">
         <is>
           <t>מודל PTT (tap+VAD) + טריגר כפתור פיזי (Pico HID→F13)</t>
         </is>
       </c>
-      <c r="D37" s="50" t="n">
+      <c r="D38" s="50" t="n">
         <v>46187</v>
       </c>
-      <c r="E37" s="50" t="n">
+      <c r="E38" s="50" t="n">
         <v>46201</v>
       </c>
-      <c r="F37" s="47">
+      <c r="F38" s="47">
         <f>E36-D36+1</f>
         <v/>
       </c>
-      <c r="G37" s="51" t="inlineStr">
+      <c r="G38" s="51" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H37" s="49" t="inlineStr">
+      <c r="H38" s="49" t="inlineStr">
         <is>
           <t>ליבה אומתה e2e 14.6: החלטה tap-to-open + VAD סוגר (לא hold). arcade button → Pico 2W (CircuitPython 10.2.1) → HID keystroke F13 → keydown ב-app.js (bindDisplayHotkeys, ענף else-if) → send(start_listening). אומת עם jumper GP21↔GND; Tico עבר ל-listening. רכיבים הוזמנו מ-Ali (~שבועיים): כפתור 30mm 5V clear ×10 · amber LED 5V prewired · טרנזיסטורים · נגדים · breadboard · jumpers. נותר: הרכבת כפתור כשמגיע · שכבת LED מונעת-מצב (GP16+טרנזיסטור, קוד מוכן) · commit app.js. אותו דפוס keystroke→WS פותח גם טריגר פיזי ל-takeaway (משימה 32).</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="40">
-      <c r="A38" s="57" t="n">
+    <row r="39" ht="15" customHeight="1" s="40">
+      <c r="A39" s="57" t="n">
         <v>30</v>
       </c>
-      <c r="B38" s="58" t="inlineStr">
+      <c r="B39" s="58" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C38" s="59" t="inlineStr">
+      <c r="C39" s="59" t="inlineStr">
         <is>
           <t>demo-mode לנפילת רשת (fallback ל-6 APIs)</t>
         </is>
       </c>
-      <c r="D38" s="60" t="n">
+      <c r="D39" s="60" t="n">
         <v>46193</v>
       </c>
-      <c r="E38" s="60" t="n">
+      <c r="E39" s="60" t="n">
         <v>46208</v>
       </c>
-      <c r="F38" s="57">
+      <c r="F39" s="57">
         <f>E37-D37+1</f>
         <v/>
       </c>
-      <c r="G38" s="61" t="inlineStr">
+      <c r="G39" s="61" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H38" s="59" t="inlineStr">
+      <c r="H39" s="59" t="inlineStr">
         <is>
           <t>חובה — קו סלולרי בודד</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1" s="40">
-      <c r="A39" s="47" t="n">
-        <v>31</v>
-      </c>
-      <c r="B39" s="48" t="inlineStr">
+    <row r="40" ht="15" customHeight="1" s="40">
+      <c r="A40" s="57" t="inlineStr">
+        <is>
+          <t>30b</t>
+        </is>
+      </c>
+      <c r="B40" s="58" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C39" s="49" t="inlineStr">
-        <is>
-          <t>attract-loop + תוכן שיחה לקהל</t>
-        </is>
-      </c>
-      <c r="D39" s="50" t="n">
-        <v>46204</v>
-      </c>
-      <c r="E39" s="50" t="n">
-        <v>46215</v>
-      </c>
-      <c r="F39" s="47">
-        <f>E38-D38+1</f>
-        <v/>
-      </c>
-      <c r="G39" s="51" t="inlineStr">
-        <is>
-          <t>CONTENT</t>
-        </is>
-      </c>
-      <c r="H39" s="49" t="inlineStr">
-        <is>
-          <t>edge cases · תשובות ל-100–200 מבקרים</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="40">
-      <c r="A40" s="57" t="n">
-        <v>32</v>
-      </c>
-      <c r="B40" s="58" t="inlineStr">
-        <is>
-          <t>אפליקציה</t>
-        </is>
-      </c>
       <c r="C40" s="59" t="inlineStr">
         <is>
-          <t>שליחת מסלול שנבנה למבקר (QR → PDF)</t>
+          <t>silence-fill UX (אינדיקציה ב-multi-tool turns)</t>
         </is>
       </c>
       <c r="D40" s="60" t="n">
-        <v>46188</v>
+        <v>46209</v>
       </c>
       <c r="E40" s="60" t="n">
-        <v>46196</v>
-      </c>
-      <c r="F40" s="57">
-        <f>E39-D39+1</f>
-        <v/>
-      </c>
+        <v>46217</v>
+      </c>
+      <c r="F40" s="57" t="n"/>
       <c r="G40" s="61" t="inlineStr">
         <is>
           <t>DEV</t>
@@ -1928,13 +1928,13 @@
       </c>
       <c r="H40" s="59" t="inlineStr">
         <is>
-          <t>שכבת must-have הושלמה ואומתה e2e (generate_takeaway→R2→QR→PDF). email נהרג (PII). נותר: trigger דרך Stream Deck + commit</t>
+          <t>שתיקה נקראת כתקלה - בעיית UX אמיתית</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="40">
       <c r="A41" s="47" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B41" s="48" t="inlineStr">
         <is>
@@ -1943,842 +1943,1197 @@
       </c>
       <c r="C41" s="49" t="inlineStr">
         <is>
-          <t>אסטרטגיית תקציב TTS (שדרוג מ-NO_TTS)</t>
+          <t>attract-loop + תוכן שיחה לקהל</t>
         </is>
       </c>
       <c r="D41" s="50" t="n">
-        <v>46208</v>
+        <v>46204</v>
       </c>
       <c r="E41" s="50" t="n">
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="F41" s="47">
-        <f>E40-D40+1</f>
+        <f>E38-D38+1</f>
         <v/>
       </c>
       <c r="G41" s="51" t="inlineStr">
         <is>
-          <t>KEY</t>
-        </is>
-      </c>
-      <c r="H41" s="49" t="n"/>
+          <t>CONTENT</t>
+        </is>
+      </c>
+      <c r="H41" s="49" t="inlineStr">
+        <is>
+          <t>edge cases · תשובות ל-100–200 מבקרים</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="40">
       <c r="A42" s="57" t="n">
+        <v>32</v>
+      </c>
+      <c r="B42" s="58" t="inlineStr">
+        <is>
+          <t>אפליקציה</t>
+        </is>
+      </c>
+      <c r="C42" s="59" t="inlineStr">
+        <is>
+          <t>שליחת מסלול שנבנה למבקר (QR → PDF)</t>
+        </is>
+      </c>
+      <c r="D42" s="60" t="n">
+        <v>46188</v>
+      </c>
+      <c r="E42" s="60" t="n">
+        <v>46196</v>
+      </c>
+      <c r="F42" s="57">
+        <f>E39-D39+1</f>
+        <v/>
+      </c>
+      <c r="G42" s="61" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+      <c r="H42" s="59" t="inlineStr">
+        <is>
+          <t>שכבת must-have הושלמה ואומתה e2e (generate_takeaway→R2→QR→PDF). email נהרג (PII). נותר: trigger דרך Stream Deck + commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="14.25" customHeight="1" s="40">
+      <c r="A43" s="57" t="inlineStr">
+        <is>
+          <t>32b</t>
+        </is>
+      </c>
+      <c r="B43" s="58" t="inlineStr">
+        <is>
+          <t>אפליקציה</t>
+        </is>
+      </c>
+      <c r="C43" s="59" t="inlineStr">
+        <is>
+          <t>QL-800 label+QR (brother_ql/CUPS)</t>
+        </is>
+      </c>
+      <c r="D43" s="60" t="n">
+        <v>46210</v>
+      </c>
+      <c r="E43" s="60" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F43" s="57" t="n"/>
+      <c r="G43" s="61" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+      <c r="H43" s="59" t="inlineStr">
+        <is>
+          <t>מנדטורי - אפס קוד; trigger ב-takeaway</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1" s="40">
+      <c r="A44" s="47" t="n">
+        <v>33</v>
+      </c>
+      <c r="B44" s="48" t="inlineStr">
+        <is>
+          <t>אפליקציה</t>
+        </is>
+      </c>
+      <c r="C44" s="49" t="inlineStr">
+        <is>
+          <t>אסטרטגיית תקציב TTS (שדרוג מ-NO_TTS)</t>
+        </is>
+      </c>
+      <c r="D44" s="50" t="n">
+        <v>46208</v>
+      </c>
+      <c r="E44" s="50" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F44" s="47">
+        <f>E40-D40+1</f>
+        <v/>
+      </c>
+      <c r="G44" s="51" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="H44" s="49" t="n"/>
+    </row>
+    <row r="45" ht="15" customHeight="1" s="40">
+      <c r="A45" s="57" t="n">
         <v>34</v>
       </c>
-      <c r="B42" s="58" t="inlineStr">
+      <c r="B45" s="58" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C42" s="59" t="inlineStr">
+      <c r="C45" s="59" t="inlineStr">
         <is>
           <t>(אופ') מנגנון interrupt "תעצור"/barge-in</t>
         </is>
       </c>
-      <c r="D42" s="60" t="n">
+      <c r="D45" s="60" t="n">
         <v>46211</v>
       </c>
-      <c r="E42" s="60" t="n">
+      <c r="E45" s="60" t="n">
         <v>46218</v>
       </c>
-      <c r="F42" s="57">
+      <c r="F45" s="57">
         <f>E41-D41+1</f>
         <v/>
       </c>
-      <c r="G42" s="61" t="inlineStr">
+      <c r="G45" s="61" t="inlineStr">
         <is>
           <t>DEV</t>
         </is>
       </c>
-      <c r="H42" s="59" t="inlineStr">
+      <c r="H45" s="59" t="inlineStr">
         <is>
           <t>נדחה; רלוונטי לקהל חי</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="14.25" customHeight="1" s="40">
-      <c r="A43" s="47" t="n">
+    <row r="46" ht="15" customHeight="1" s="40">
+      <c r="A46" s="47" t="n">
         <v>35</v>
       </c>
-      <c r="B43" s="48" t="inlineStr">
+      <c r="B46" s="48" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C43" s="49" t="inlineStr">
+      <c r="C46" s="49" t="inlineStr">
         <is>
           <t>QA אינטגרציה מלאה (כל הסוכנים e2e)</t>
         </is>
       </c>
-      <c r="D43" s="50" t="n">
+      <c r="D46" s="50" t="n">
         <v>46216</v>
       </c>
-      <c r="E43" s="50" t="n">
+      <c r="E46" s="50" t="n">
         <v>46225</v>
       </c>
-      <c r="F43" s="47">
+      <c r="F46" s="47">
         <f>E42-D42+1</f>
         <v/>
       </c>
-      <c r="G43" s="51" t="inlineStr">
+      <c r="G46" s="51" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="H43" s="49" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="40">
-      <c r="A44" s="57" t="n">
+      <c r="H46" s="49" t="n"/>
+    </row>
+    <row r="47" ht="15" customHeight="1" s="40">
+      <c r="A47" s="57" t="n">
         <v>36</v>
       </c>
-      <c r="B44" s="58" t="inlineStr">
+      <c r="B47" s="58" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C44" s="59" t="inlineStr">
+      <c r="C47" s="59" t="inlineStr">
         <is>
           <t>pilot עם משתמשים אמיתיים</t>
         </is>
       </c>
-      <c r="D44" s="60" t="n">
+      <c r="D47" s="60" t="n">
         <v>46225</v>
       </c>
-      <c r="E44" s="60" t="n">
+      <c r="E47" s="60" t="n">
         <v>46231</v>
       </c>
-      <c r="F44" s="57">
+      <c r="F47" s="57">
         <f>E43-D43+1</f>
         <v/>
       </c>
-      <c r="G44" s="61" t="inlineStr">
+      <c r="G47" s="61" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H44" s="59" t="inlineStr">
+      <c r="H47" s="59" t="inlineStr">
         <is>
           <t>לגלות הפתעות לפני קהל</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1" s="40">
-      <c r="A45" s="47" t="n">
+    <row r="48" ht="15" customHeight="1" s="40">
+      <c r="A48" s="47" t="n">
         <v>37</v>
       </c>
-      <c r="B45" s="48" t="inlineStr">
+      <c r="B48" s="48" t="inlineStr">
         <is>
           <t>אפליקציה</t>
         </is>
       </c>
-      <c r="C45" s="49" t="inlineStr">
+      <c r="C48" s="49" t="inlineStr">
         <is>
           <t>watchdog/auto-relaunch לריצה רציפה 14 ימים</t>
         </is>
       </c>
-      <c r="D45" s="50" t="n">
+      <c r="D48" s="50" t="n">
         <v>46198</v>
       </c>
-      <c r="E45" s="50" t="n">
+      <c r="E48" s="50" t="n">
         <v>46211</v>
       </c>
-      <c r="F45" s="47" t="n"/>
-      <c r="G45" s="51" t="inlineStr">
+      <c r="F48" s="47" t="n"/>
+      <c r="G48" s="51" t="inlineStr">
         <is>
           <t>DEV</t>
         </is>
       </c>
-      <c r="H45" s="49" t="inlineStr">
+      <c r="H48" s="49" t="inlineStr">
         <is>
           <t>אם הדמו קורס בלילה בריצה לא-מאוישת — זיהוי + הפעלה-מחדש אוטומטית · ⚠ טרם התחיל — אפס artifacts (deploy+אמינות 14 יום); תאריך מיושן</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="15" customHeight="1" s="40">
-      <c r="A46" s="57" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="40">
-      <c r="A47" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  תערוכה / לוגיסטיקה — Exhibition</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="40">
-      <c r="A48" s="57" t="n">
-        <v>39</v>
-      </c>
-      <c r="B48" s="58" t="inlineStr">
-        <is>
-          <t>תערוכה</t>
-        </is>
-      </c>
-      <c r="C48" s="59" t="inlineStr">
-        <is>
-          <t>✅ החלטות חלל/מיצב</t>
-        </is>
-      </c>
-      <c r="D48" s="60" t="n">
-        <v>46171</v>
-      </c>
-      <c r="E48" s="60" t="n">
-        <v>46171</v>
-      </c>
-      <c r="F48" s="57">
-        <f>E45-D45+1</f>
-        <v/>
-      </c>
-      <c r="G48" s="61" t="inlineStr">
+    <row r="49" ht="15" customHeight="1" s="40">
+      <c r="A49" s="47" t="inlineStr">
+        <is>
+          <t>37b</t>
+        </is>
+      </c>
+      <c r="B49" s="48" t="inlineStr">
+        <is>
+          <t>אפליקציה</t>
+        </is>
+      </c>
+      <c r="C49" s="49" t="inlineStr">
+        <is>
+          <t>soak 14 יום ללא השגחה (heartbeat+watchdog)</t>
+        </is>
+      </c>
+      <c r="D49" s="50" t="n">
+        <v>46212</v>
+      </c>
+      <c r="E49" s="50" t="n">
+        <v>46226</v>
+      </c>
+      <c r="F49" s="47" t="n"/>
+      <c r="G49" s="51" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H48" s="59" t="inlineStr">
-        <is>
-          <t>מסך אחד · handset+PTT · Stream Deck Neo</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="40">
-      <c r="A49" s="47" t="n">
-        <v>40</v>
-      </c>
-      <c r="B49" s="48" t="inlineStr">
-        <is>
-          <t>תערוכה</t>
-        </is>
-      </c>
-      <c r="C49" s="49" t="inlineStr">
-        <is>
-          <t>קבלת spec מ-HIT</t>
-        </is>
-      </c>
-      <c r="D49" s="50" t="n">
-        <v>46174</v>
-      </c>
-      <c r="E49" s="50" t="n">
-        <v>46183</v>
-      </c>
-      <c r="F49" s="47">
-        <f>E46-D46+1</f>
-        <v/>
-      </c>
-      <c r="G49" s="51" t="inlineStr">
-        <is>
-          <t>KEY</t>
-        </is>
-      </c>
       <c r="H49" s="49" t="inlineStr">
         <is>
-          <t>היה ל-26.5, מאחר — חוסם פרק 7/מיפוי/חשמל</t>
+          <t>סיכון 1 - אפס artifacts; הריצה עצמה לא ה-harness (37)</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="40">
-      <c r="A50" s="57" t="n">
-        <v>41</v>
-      </c>
-      <c r="B50" s="58" t="inlineStr">
-        <is>
-          <t>תערוכה</t>
-        </is>
-      </c>
-      <c r="C50" s="59" t="inlineStr">
-        <is>
-          <t>קביעת דגם Mac mini + גודל מסך</t>
-        </is>
-      </c>
-      <c r="D50" s="60" t="n">
-        <v>46176</v>
-      </c>
-      <c r="E50" s="60" t="n">
-        <v>46183</v>
-      </c>
-      <c r="F50" s="57">
-        <f>E47-D47+1</f>
-        <v/>
-      </c>
-      <c r="G50" s="61" t="inlineStr">
-        <is>
-          <t>HW</t>
-        </is>
-      </c>
-      <c r="H50" s="59" t="inlineStr">
-        <is>
-          <t>לחישוב חשמל מדויק</t>
-        </is>
-      </c>
+      <c r="A50" s="57" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="40">
-      <c r="A51" s="47" t="n">
-        <v>42</v>
-      </c>
-      <c r="B51" s="48" t="inlineStr">
-        <is>
-          <t>תערוכה</t>
-        </is>
-      </c>
-      <c r="C51" s="49" t="inlineStr">
-        <is>
-          <t>החלטת גיבוי חומרה (Mac mini/מודם/מיק רזרבי)</t>
-        </is>
-      </c>
-      <c r="D51" s="50" t="n">
-        <v>46185</v>
-      </c>
-      <c r="E51" s="50" t="n">
-        <v>46193</v>
-      </c>
-      <c r="F51" s="47" t="n"/>
-      <c r="G51" s="51" t="inlineStr">
-        <is>
-          <t>HW</t>
-        </is>
-      </c>
-      <c r="H51" s="49" t="inlineStr">
-        <is>
-          <t>מה קורה אם רכיב נופל באמצע 14 הימים — להחליט על רזרבה לפני התערוכה</t>
+      <c r="A51" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  סרטון Hero + מסך הדמיות — Video</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="40">
-      <c r="A52" s="57" t="n">
-        <v>43</v>
+      <c r="A52" s="57" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
       </c>
       <c r="B52" s="58" t="inlineStr">
         <is>
-          <t>תערוכה</t>
+          <t>סרטון</t>
         </is>
       </c>
       <c r="C52" s="59" t="inlineStr">
         <is>
-          <t>קבלת מודם סלולרי</t>
+          <t>פרומפטים סופיים + עוגן-Maya + P1/P9b -&gt; נעילת reference</t>
         </is>
       </c>
       <c r="D52" s="60" t="n">
-        <v>46185</v>
+        <v>46203</v>
       </c>
       <c r="E52" s="60" t="n">
-        <v>46185</v>
-      </c>
-      <c r="F52" s="57">
-        <f>E48-D48+1</f>
-        <v/>
-      </c>
+        <v>46206</v>
+      </c>
+      <c r="F52" s="57" t="n"/>
       <c r="G52" s="61" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>DESIGN</t>
         </is>
       </c>
       <c r="H52" s="59" t="inlineStr">
         <is>
-          <t>~שבועיים — חוסם בדיקת demo-mode</t>
+          <t>Grok - composite-Tico; השער לפני פאנלים</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="40">
-      <c r="A53" s="47" t="n">
-        <v>44</v>
-      </c>
-      <c r="B53" s="48" t="inlineStr">
-        <is>
-          <t>תערוכה</t>
-        </is>
-      </c>
-      <c r="C53" s="49" t="inlineStr">
-        <is>
-          <t>מיפוי סופי + אישור חשמל/UPS מול האוצרת</t>
-        </is>
-      </c>
-      <c r="D53" s="50" t="n">
-        <v>46195</v>
-      </c>
-      <c r="E53" s="50" t="n">
-        <v>46201</v>
-      </c>
-      <c r="F53" s="47">
-        <f>E49-D49+1</f>
-        <v/>
-      </c>
-      <c r="G53" s="51" t="inlineStr">
-        <is>
-          <t>KEY</t>
-        </is>
-      </c>
-      <c r="H53" s="49" t="inlineStr">
-        <is>
-          <t>שקע 230V מוארק ייעודי + UPS קטן</t>
+      <c r="A53" s="57" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B53" s="58" t="inlineStr">
+        <is>
+          <t>סרטון</t>
+        </is>
+      </c>
+      <c r="C53" s="59" t="inlineStr">
+        <is>
+          <t>אנימטיק (VO-draft + תזמון Premiere)</t>
+        </is>
+      </c>
+      <c r="D53" s="60" t="n">
+        <v>46206</v>
+      </c>
+      <c r="E53" s="60" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F53" s="57" t="n"/>
+      <c r="G53" s="61" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="H53" s="59" t="inlineStr">
+        <is>
+          <t>לפני ייצור - חוסך רנדרים (Grok 6/10ש לא חותכים)</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="40">
-      <c r="A54" s="57" t="n">
-        <v>45</v>
+      <c r="A54" s="57" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
       </c>
       <c r="B54" s="58" t="inlineStr">
         <is>
-          <t>תערוכה</t>
+          <t>סרטון</t>
         </is>
       </c>
       <c r="C54" s="59" t="inlineStr">
         <is>
-          <t>בדיקת תנאי-אמת Mac mini בחלל</t>
+          <t>ייצור 16 פאנלים + הרכבת Tico (glow-&gt;וקטור)</t>
         </is>
       </c>
       <c r="D54" s="60" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="E54" s="60" t="n">
         <v>46215</v>
       </c>
-      <c r="F54" s="57">
+      <c r="F54" s="57" t="n"/>
+      <c r="G54" s="61" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="H54" s="59" t="inlineStr">
+        <is>
+          <t>לפי אורכי האנימטיק</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15" customHeight="1" s="40">
+      <c r="A55" s="57" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="B55" s="58" t="inlineStr">
+        <is>
+          <t>סרטון</t>
+        </is>
+      </c>
+      <c r="C55" s="59" t="inlineStr">
+        <is>
+          <t>שתילה ב-storyboard + ייצוא PDF למנחה</t>
+        </is>
+      </c>
+      <c r="D55" s="60" t="n">
+        <v>46215</v>
+      </c>
+      <c r="E55" s="60" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F55" s="57" t="n"/>
+      <c r="G55" s="61" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="H55" s="59" t="inlineStr">
+        <is>
+          <t>deliverable למנחה</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15" customHeight="1" s="40">
+      <c r="A56" s="57" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="B56" s="58" t="inlineStr">
+        <is>
+          <t>סרטון</t>
+        </is>
+      </c>
+      <c r="C56" s="59" t="inlineStr">
+        <is>
+          <t>מסך הדמיות 3 - build (וידאו-לופ + 2-3 סימולציות)</t>
+        </is>
+      </c>
+      <c r="D56" s="60" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E56" s="60" t="n">
+        <v>46225</v>
+      </c>
+      <c r="F56" s="57" t="n"/>
+      <c r="G56" s="61" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+      <c r="H56" s="59" t="inlineStr">
+        <is>
+          <t>חסום על החלטת תוכן: build-route/לוח/takeaway</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15" customHeight="1" s="40">
+      <c r="A57" s="57" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="58" ht="15" customHeight="1" s="40">
+      <c r="A58" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  תערוכה / לוגיסטיקה — Exhibition</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1" s="40">
+      <c r="A59" s="57" t="n">
+        <v>39</v>
+      </c>
+      <c r="B59" s="58" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C59" s="59" t="inlineStr">
+        <is>
+          <t>✅ החלטות חלל/מיצב</t>
+        </is>
+      </c>
+      <c r="D59" s="60" t="n">
+        <v>46171</v>
+      </c>
+      <c r="E59" s="60" t="n">
+        <v>46171</v>
+      </c>
+      <c r="F59" s="57">
+        <f>E45-D45+1</f>
+        <v/>
+      </c>
+      <c r="G59" s="61" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="H59" s="59" t="inlineStr">
+        <is>
+          <t>מסך אחד · handset+PTT · Stream Deck Neo</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15" customHeight="1" s="40">
+      <c r="A60" s="47" t="n">
+        <v>40</v>
+      </c>
+      <c r="B60" s="48" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C60" s="49" t="inlineStr">
+        <is>
+          <t>קבלת spec מ-HIT</t>
+        </is>
+      </c>
+      <c r="D60" s="50" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E60" s="50" t="n">
+        <v>46183</v>
+      </c>
+      <c r="F60" s="47">
+        <f>E46-D46+1</f>
+        <v/>
+      </c>
+      <c r="G60" s="51" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="H60" s="49" t="inlineStr">
+        <is>
+          <t>היה ל-26.5, מאחר — חוסם פרק 7/מיפוי/חשמל</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15" customHeight="1" s="40">
+      <c r="A61" s="57" t="n">
+        <v>41</v>
+      </c>
+      <c r="B61" s="58" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C61" s="59" t="inlineStr">
+        <is>
+          <t>קביעת דגם Mac mini + גודל מסך</t>
+        </is>
+      </c>
+      <c r="D61" s="60" t="n">
+        <v>46176</v>
+      </c>
+      <c r="E61" s="60" t="n">
+        <v>46183</v>
+      </c>
+      <c r="F61" s="57">
+        <f>E47-D47+1</f>
+        <v/>
+      </c>
+      <c r="G61" s="61" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+      <c r="H61" s="59" t="inlineStr">
+        <is>
+          <t>לחישוב חשמל מדויק</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15" customHeight="1" s="40">
+      <c r="A62" s="47" t="n">
+        <v>42</v>
+      </c>
+      <c r="B62" s="48" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C62" s="49" t="inlineStr">
+        <is>
+          <t>החלטת גיבוי חומרה (Mac mini/מודם/מיק רזרבי)</t>
+        </is>
+      </c>
+      <c r="D62" s="50" t="n">
+        <v>46185</v>
+      </c>
+      <c r="E62" s="50" t="n">
+        <v>46193</v>
+      </c>
+      <c r="F62" s="47" t="n"/>
+      <c r="G62" s="51" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+      <c r="H62" s="49" t="inlineStr">
+        <is>
+          <t>מה קורה אם רכיב נופל באמצע 14 הימים — להחליט על רזרבה לפני התערוכה</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15" customHeight="1" s="40">
+      <c r="A63" s="57" t="n">
+        <v>43</v>
+      </c>
+      <c r="B63" s="58" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C63" s="59" t="inlineStr">
+        <is>
+          <t>קבלת מודם סלולרי</t>
+        </is>
+      </c>
+      <c r="D63" s="60" t="n">
+        <v>46185</v>
+      </c>
+      <c r="E63" s="60" t="n">
+        <v>46185</v>
+      </c>
+      <c r="F63" s="57">
+        <f>E48-D48+1</f>
+        <v/>
+      </c>
+      <c r="G63" s="61" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+      <c r="H63" s="59" t="inlineStr">
+        <is>
+          <t>~שבועיים — חוסם בדיקת demo-mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15" customHeight="1" s="40">
+      <c r="A64" s="47" t="n">
+        <v>44</v>
+      </c>
+      <c r="B64" s="48" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C64" s="49" t="inlineStr">
+        <is>
+          <t>מיפוי סופי + אישור חשמל/UPS מול האוצרת</t>
+        </is>
+      </c>
+      <c r="D64" s="50" t="n">
+        <v>46195</v>
+      </c>
+      <c r="E64" s="50" t="n">
+        <v>46201</v>
+      </c>
+      <c r="F64" s="47">
+        <f>E49-D49+1</f>
+        <v/>
+      </c>
+      <c r="G64" s="51" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="H64" s="49" t="inlineStr">
+        <is>
+          <t>שקע 230V מוארק ייעודי + UPS קטן</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="15" customHeight="1" s="40">
+      <c r="A65" s="57" t="n">
+        <v>45</v>
+      </c>
+      <c r="B65" s="58" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C65" s="59" t="inlineStr">
+        <is>
+          <t>בדיקת תנאי-אמת Mac mini בחלל</t>
+        </is>
+      </c>
+      <c r="D65" s="60" t="n">
+        <v>46209</v>
+      </c>
+      <c r="E65" s="60" t="n">
+        <v>46215</v>
+      </c>
+      <c r="F65" s="57">
         <f>E50-D50+1</f>
         <v/>
       </c>
-      <c r="G54" s="61" t="inlineStr">
+      <c r="G65" s="61" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H54" s="59" t="inlineStr">
+      <c r="H65" s="59" t="inlineStr">
         <is>
           <t>מומלץ למשוך קדימה — לא להשאיר לסוף יולי</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="15" customHeight="1" s="40">
-      <c r="A55" s="47" t="n">
+    <row r="66" ht="15" customHeight="1" s="40">
+      <c r="A66" s="47" t="n">
         <v>46</v>
       </c>
-      <c r="B55" s="48" t="inlineStr">
+      <c r="B66" s="48" t="inlineStr">
         <is>
           <t>תערוכה</t>
         </is>
       </c>
-      <c r="C55" s="49" t="inlineStr">
+      <c r="C66" s="49" t="inlineStr">
         <is>
           <t>עיצוב פוסטר 1×0.7 (פורטרט)</t>
         </is>
       </c>
-      <c r="D55" s="50" t="n">
+      <c r="D66" s="50" t="n">
         <v>46204</v>
       </c>
-      <c r="E55" s="50" t="n">
+      <c r="E66" s="50" t="n">
         <v>46213</v>
       </c>
-      <c r="F55" s="47">
+      <c r="F66" s="47">
         <f>E51-D51+1</f>
         <v/>
       </c>
-      <c r="G55" s="51" t="inlineStr">
+      <c r="G66" s="51" t="inlineStr">
         <is>
           <t>DESIGN</t>
         </is>
       </c>
-      <c r="H55" s="49" t="n"/>
-    </row>
-    <row r="56" ht="15" customHeight="1" s="40">
-      <c r="A56" s="57" t="n">
+      <c r="H66" s="49" t="n"/>
+    </row>
+    <row r="67" ht="15" customHeight="1" s="40">
+      <c r="A67" s="57" t="n">
         <v>47</v>
       </c>
-      <c r="B56" s="58" t="inlineStr">
+      <c r="B67" s="58" t="inlineStr">
         <is>
           <t>תערוכה</t>
         </is>
       </c>
-      <c r="C56" s="59" t="inlineStr">
+      <c r="C67" s="59" t="inlineStr">
         <is>
           <t>QR/הדפסת מסלול — takeaway פיזי למבקר</t>
         </is>
       </c>
-      <c r="D56" s="60" t="n">
+      <c r="D67" s="60" t="n">
         <v>46216</v>
       </c>
-      <c r="E56" s="60" t="n">
+      <c r="E67" s="60" t="n">
         <v>46219</v>
       </c>
-      <c r="F56" s="57">
+      <c r="F67" s="57">
         <f>E52-D52+1</f>
         <v/>
       </c>
-      <c r="G56" s="61" t="inlineStr">
+      <c r="G67" s="61" t="inlineStr">
         <is>
           <t>DEV</t>
         </is>
       </c>
-      <c r="H56" s="59" t="inlineStr">
+      <c r="H67" s="59" t="inlineStr">
         <is>
           <t>פריסת הדפסה/QR; תלוי בפיצ'ר ה-export (משימה 32) · QL-800 label — אפס קוד, מנדטורי, בנייה מאפס</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="14.25" customHeight="1" s="40">
-      <c r="A57" s="47" t="n">
+    <row r="68">
+      <c r="A68" s="47" t="inlineStr">
+        <is>
+          <t>Bd</t>
+        </is>
+      </c>
+      <c r="B68" s="48" t="inlineStr">
+        <is>
+          <t>תערוכה</t>
+        </is>
+      </c>
+      <c r="C68" s="49" t="inlineStr">
+        <is>
+          <t>תיקון bidi בלוח (bdi + הסרת em-dashes ש 372-403)</t>
+        </is>
+      </c>
+      <c r="D68" s="50" t="n">
+        <v>46204</v>
+      </c>
+      <c r="E68" s="50" t="n">
+        <v>46206</v>
+      </c>
+      <c r="F68" s="47" t="n"/>
+      <c r="G68" s="51" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="H68" s="49" t="inlineStr">
+        <is>
+          <t>docs/samples/odysee-board-v1.html - ישיבה אחת</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="47" t="n">
         <v>48</v>
       </c>
-      <c r="B57" s="48" t="inlineStr">
+      <c r="B69" s="48" t="inlineStr">
         <is>
           <t>תערוכה</t>
         </is>
       </c>
-      <c r="C57" s="49" t="inlineStr">
+      <c r="C69" s="49" t="inlineStr">
         <is>
           <t>הדפסת פוסטר + חומרי הסבר</t>
         </is>
       </c>
-      <c r="D57" s="50" t="n">
+      <c r="D69" s="50" t="n">
         <v>46223</v>
       </c>
-      <c r="E57" s="50" t="n">
+      <c r="E69" s="50" t="n">
         <v>46229</v>
       </c>
-      <c r="F57" s="47">
+      <c r="F69" s="47">
         <f>E53-D53+1</f>
         <v/>
       </c>
-      <c r="G57" s="51" t="inlineStr">
+      <c r="G69" s="51" t="inlineStr">
         <is>
           <t>PRINT</t>
         </is>
       </c>
-      <c r="H57" s="49" t="n"/>
-    </row>
-    <row r="58" ht="15" customHeight="1" s="40">
-      <c r="A58" s="57" t="n">
+      <c r="H69" s="49" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="57" t="n">
         <v>49</v>
       </c>
-      <c r="B58" s="58" t="inlineStr">
+      <c r="B70" s="58" t="inlineStr">
         <is>
           <t>תערוכה</t>
         </is>
       </c>
-      <c r="C58" s="59" t="inlineStr">
+      <c r="C70" s="59" t="inlineStr">
         <is>
           <t>הרכבת חומרה + בדיקות</t>
         </is>
       </c>
-      <c r="D58" s="60" t="n">
+      <c r="D70" s="60" t="n">
         <v>46231</v>
       </c>
-      <c r="E58" s="60" t="n">
+      <c r="E70" s="60" t="n">
         <v>46237</v>
       </c>
-      <c r="F58" s="57">
+      <c r="F70" s="57">
         <f>E54-D54+1</f>
         <v/>
       </c>
-      <c r="G58" s="61" t="inlineStr">
+      <c r="G70" s="61" t="inlineStr">
         <is>
           <t>HW</t>
         </is>
       </c>
-      <c r="H58" s="59" t="inlineStr">
+      <c r="H70" s="59" t="inlineStr">
         <is>
           <t>מסך · רמקול · מיקרופון · Stream Deck</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="15" customHeight="1" s="40">
-      <c r="A59" s="47" t="n">
+    <row r="71">
+      <c r="A71" s="47" t="n">
         <v>50</v>
       </c>
-      <c r="B59" s="48" t="inlineStr">
+      <c r="B71" s="48" t="inlineStr">
         <is>
           <t>תערוכה</t>
         </is>
       </c>
-      <c r="C59" s="49" t="inlineStr">
+      <c r="C71" s="49" t="inlineStr">
         <is>
           <t>הקמת התערוכה בחלל</t>
         </is>
       </c>
-      <c r="D59" s="50" t="n">
+      <c r="D71" s="50" t="n">
         <v>46239</v>
       </c>
-      <c r="E59" s="50" t="n">
+      <c r="E71" s="50" t="n">
         <v>46239</v>
       </c>
-      <c r="F59" s="47">
+      <c r="F71" s="47">
         <f>E55-D55+1</f>
         <v/>
       </c>
-      <c r="G59" s="51" t="inlineStr">
+      <c r="G71" s="51" t="inlineStr">
         <is>
           <t>SETUP</t>
         </is>
       </c>
-      <c r="H59" s="49" t="inlineStr">
+      <c r="H71" s="49" t="inlineStr">
         <is>
           <t>התקנה + בדיקה סופית במקום</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="15" customHeight="1" s="40">
-      <c r="A60" s="57" t="n">
+    <row r="72">
+      <c r="A72" s="57" t="n">
         <v>51</v>
       </c>
-      <c r="B60" s="58" t="inlineStr">
+      <c r="B72" s="58" t="inlineStr">
         <is>
           <t>תערוכה</t>
         </is>
       </c>
-      <c r="C60" s="59" t="inlineStr">
+      <c r="C72" s="59" t="inlineStr">
         <is>
           <t>ימי תערוכה + תיעוד מערכת חיה</t>
         </is>
       </c>
-      <c r="D60" s="60" t="n">
+      <c r="D72" s="60" t="n">
         <v>46240</v>
       </c>
-      <c r="E60" s="60" t="n">
+      <c r="E72" s="60" t="n">
         <v>46253</v>
       </c>
-      <c r="F60" s="57">
+      <c r="F72" s="57">
         <f>E56-D56+1</f>
         <v/>
       </c>
-      <c r="G60" s="61" t="inlineStr">
+      <c r="G72" s="61" t="inlineStr">
         <is>
           <t>LIVE</t>
         </is>
       </c>
-      <c r="H60" s="59" t="inlineStr">
+      <c r="H72" s="59" t="inlineStr">
         <is>
           <t>וידאו+סטילס · הפעלה יומית · feedback</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="15" customHeight="1" s="40">
-      <c r="A61" s="47" t="n">
+    <row r="73">
+      <c r="A73" s="47" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="62" ht="15" customHeight="1" s="40">
-      <c r="A62" s="46" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">  אבני דרך — Milestones</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="15" customHeight="1" s="40">
-      <c r="A63" s="47" t="n">
+    <row r="75">
+      <c r="A75" s="47" t="n">
         <v>53</v>
       </c>
-      <c r="B63" s="48" t="inlineStr">
+      <c r="B75" s="48" t="inlineStr">
         <is>
           <t>אבן דרך</t>
         </is>
       </c>
-      <c r="C63" s="49" t="inlineStr">
+      <c r="C75" s="49" t="inlineStr">
         <is>
           <t>📌 פגישת מנחה</t>
         </is>
       </c>
-      <c r="D63" s="50" t="n">
+      <c r="D75" s="50" t="n">
         <v>46175</v>
       </c>
-      <c r="E63" s="50" t="n">
+      <c r="E75" s="50" t="n">
         <v>46175</v>
       </c>
-      <c r="F63" s="47">
+      <c r="F75" s="47">
         <f>E59-D59+1</f>
         <v/>
       </c>
-      <c r="G63" s="51" t="inlineStr">
+      <c r="G75" s="51" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H63" s="49" t="inlineStr">
+      <c r="H75" s="49" t="inlineStr">
         <is>
           <t>מגדיר את דרישות הצגת הביניים</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="15" customHeight="1" s="40">
-      <c r="A64" s="57" t="n">
+    <row r="76">
+      <c r="A76" s="57" t="n">
         <v>54</v>
       </c>
-      <c r="B64" s="58" t="inlineStr">
+      <c r="B76" s="58" t="inlineStr">
         <is>
           <t>אבן דרך</t>
         </is>
       </c>
-      <c r="C64" s="59" t="inlineStr">
+      <c r="C76" s="59" t="inlineStr">
         <is>
           <t>📌 הצגת ביניים</t>
         </is>
       </c>
-      <c r="D64" s="60" t="n">
+      <c r="D76" s="60" t="n">
         <v>46189</v>
       </c>
-      <c r="E64" s="60" t="n">
+      <c r="E76" s="60" t="n">
         <v>46189</v>
       </c>
-      <c r="F64" s="57">
+      <c r="F76" s="57">
         <f>E60-D60+1</f>
         <v/>
       </c>
-      <c r="G64" s="61" t="inlineStr">
+      <c r="G76" s="61" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H64" s="59" t="inlineStr">
+      <c r="H76" s="59" t="inlineStr">
         <is>
           <t>יום שלישי 16.6 · deck v10 + presenter notes מוכנים · חזרה אחרונה 15.6 ערב · האתר לא מוצג</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="15" customHeight="1" s="40">
-      <c r="A65" s="47" t="n">
+    <row r="77">
+      <c r="A77" s="47" t="n">
         <v>55</v>
       </c>
-      <c r="B65" s="48" t="inlineStr">
+      <c r="B77" s="48" t="inlineStr">
         <is>
           <t>אבן דרך</t>
         </is>
       </c>
-      <c r="C65" s="49" t="inlineStr">
+      <c r="C77" s="49" t="inlineStr">
         <is>
           <t>📌 הקפאת ספר</t>
         </is>
       </c>
-      <c r="D65" s="50" t="n">
+      <c r="D77" s="50" t="n">
         <v>46229</v>
       </c>
-      <c r="E65" s="50" t="n">
+      <c r="E77" s="50" t="n">
         <v>46229</v>
       </c>
-      <c r="F65" s="47">
+      <c r="F77" s="47">
         <f>E61-D61+1</f>
         <v/>
       </c>
-      <c r="G65" s="51" t="inlineStr">
+      <c r="G77" s="51" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H65" s="49" t="inlineStr">
+      <c r="H77" s="49" t="inlineStr">
         <is>
           <t>תוכן סופי לפני בנייה+הדפסה · גזור ל-lead-time של Zami — אמת השבוע</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="15" customHeight="1" s="40">
-      <c r="A66" s="57" t="n">
+    <row r="78">
+      <c r="A78" s="57" t="n">
         <v>56</v>
       </c>
-      <c r="B66" s="58" t="inlineStr">
+      <c r="B78" s="58" t="inlineStr">
         <is>
           <t>אבן דרך</t>
         </is>
       </c>
-      <c r="C66" s="59" t="inlineStr">
+      <c r="C78" s="59" t="inlineStr">
         <is>
           <t>📌 dry-run מלא בתנאי תערוכה</t>
         </is>
       </c>
-      <c r="D66" s="60" t="n">
+      <c r="D78" s="60" t="n">
         <v>46237</v>
       </c>
-      <c r="E66" s="60" t="n">
+      <c r="E78" s="60" t="n">
         <v>46239</v>
       </c>
-      <c r="F66" s="57">
+      <c r="F78" s="57">
         <f>E62-D62+1</f>
         <v/>
       </c>
-      <c r="G66" s="61" t="inlineStr">
+      <c r="G78" s="61" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="H66" s="59" t="inlineStr">
+      <c r="H78" s="59" t="inlineStr">
         <is>
           <t>ריצה מלאה כמו יום הפתיחה</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" s="40">
-      <c r="A67" s="47" t="n">
+    <row r="79">
+      <c r="A79" s="47" t="n">
         <v>57</v>
       </c>
-      <c r="B67" s="48" t="inlineStr">
+      <c r="B79" s="48" t="inlineStr">
         <is>
           <t>אבן דרך</t>
         </is>
       </c>
-      <c r="C67" s="49" t="inlineStr">
+      <c r="C79" s="49" t="inlineStr">
         <is>
           <t>📌 הגשת הספר</t>
         </is>
       </c>
-      <c r="D67" s="50" t="n">
+      <c r="D79" s="50" t="n">
         <v>46264</v>
       </c>
-      <c r="E67" s="50" t="n">
+      <c r="E79" s="50" t="n">
         <v>46264</v>
       </c>
-      <c r="F67" s="47">
+      <c r="F79" s="47">
         <f>E63-D63+1</f>
         <v/>
       </c>
-      <c r="G67" s="51" t="inlineStr">
+      <c r="G79" s="51" t="inlineStr">
         <is>
           <t>SUBMIT</t>
         </is>
       </c>
-      <c r="H67" s="49" t="inlineStr">
+      <c r="H79" s="49" t="inlineStr">
         <is>
           <t>דיגיטלי · 30.8 רשת ביטחון; יעד אמיתי = מודפס לפתיחה 6.8</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="57" t="n">
+    <row r="80">
+      <c r="A80" s="57" t="n">
         <v>58</v>
       </c>
-      <c r="B68" s="58" t="inlineStr">
+      <c r="B80" s="58" t="inlineStr">
         <is>
           <t>אבן דרך</t>
         </is>
       </c>
-      <c r="C68" s="59" t="inlineStr">
+      <c r="C80" s="59" t="inlineStr">
         <is>
           <t>📌 פתיחת תערוכה</t>
         </is>
       </c>
-      <c r="D68" s="60" t="n">
+      <c r="D80" s="60" t="n">
         <v>46240</v>
       </c>
-      <c r="E68" s="60" t="n">
+      <c r="E80" s="60" t="n">
         <v>46240</v>
       </c>
-      <c r="F68" s="57">
+      <c r="F80" s="57">
         <f>E64-D64+1</f>
         <v/>
       </c>
-      <c r="G68" s="61" t="inlineStr">
+      <c r="G80" s="61" t="inlineStr">
         <is>
           <t>LIVE</t>
         </is>
       </c>
-      <c r="H68" s="59" t="n"/>
+      <c r="H80" s="59" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A18:H18"/>
+  <mergeCells count="10">
+    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="A74:H74"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
plan: v4 - P12=memory-glow, Hanan board review 07.07, hero reschedule (composite 04-06.7, HD/music after), construction decision target 07.07
</commit_message>
<xml_diff>
--- a/scripts/ticoprojectplanv2.xlsx
+++ b/scripts/ticoprojectplanv2.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="187">
   <si>
     <t xml:space="preserve">Odysee — Personal AI Travel Companion · Project Plan</t>
   </si>
@@ -432,10 +432,10 @@
     <t xml:space="preserve">H3</t>
   </si>
   <si>
-    <t xml:space="preserve">🔴 החלטת P12 (iPad מול זיכרון-אור)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">חוסמת שוט 13 · החלטה תזתית (מסך=עֵד, לא נהג)</t>
+    <t xml:space="preserve">P12 = זיכרון-אור (החלטת David)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לא iPad (קו-אדום: מסך=עֵד, לא נהג) · ממתין לאישור חנן 7.7</t>
   </si>
   <si>
     <t xml:space="preserve">H4</t>
@@ -444,7 +444,7 @@
     <t xml:space="preserve">composite הסימן הווקטורי בכל שוט (Motion/AE)</t>
   </si>
   <si>
-    <t xml:space="preserve">סהרון ברוגע · פה פתוח P8 בלבד · כבוי P1 · המשימה הגדולה שנותרה</t>
+    <t xml:space="preserve">כולל שוט 13 בזיכרון-אור composited · חובה ל-6.7 · המשימה הגדולה שנותרה</t>
   </si>
   <si>
     <t xml:space="preserve">H5</t>
@@ -453,7 +453,7 @@
     <t xml:space="preserve">HD re-export P6–P10 + נרמול AR ל-16:9</t>
   </si>
   <si>
-    <t xml:space="preserve">רזולוציה נוכחית נמוכה לתערוכה</t>
+    <t xml:space="preserve">post-חנן · polish רזולוציה</t>
   </si>
   <si>
     <t xml:space="preserve">H6</t>
@@ -462,7 +462,7 @@
     <t xml:space="preserve">מוזיקה/פס-קול (~44ש שקט) + מיקס VO</t>
   </si>
   <si>
-    <t xml:space="preserve">עדיין לא פתור · VO נכנס נפרד</t>
+    <t xml:space="preserve">stretch · גרסה ראשונה עד 7.7 אם יש זמן · לא חוסם הצגת חנן · אחרת אחרי</t>
   </si>
   <si>
     <t xml:space="preserve">  תערוכה / לוגיסטיקה — Exhibition</t>
@@ -513,10 +513,10 @@
     <t xml:space="preserve">44b</t>
   </si>
   <si>
-    <t xml:space="preserve">קונסטרוקציית רקע/קיר — בהחלטה (כיוון מפושט)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">David שוקל כיוון פשוט וקל מבד-מתוח · החלטה ~יומיים · חוסם מדבקת-קיר + טופס בטיחות</t>
+    <t xml:space="preserve">קונסטרוקציית רקע/קיר — יעד החלטה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">יעד להחלטת כיוון (מפושט) · לא ביצוע · חוסם מדבקת-קיר + טופס בטיחות</t>
   </si>
   <si>
     <t xml:space="preserve">בדיקת תנאי-אמת Mac mini בחלל</t>
@@ -591,6 +591,15 @@
     <t xml:space="preserve">יום שלישי 16.6 · deck v10 + presenter notes מוכנים · חזרה אחרונה 15.6 ערב · האתר לא מוצג</t>
   </si>
   <si>
+    <t xml:space="preserve">54b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📌 הצגת video board לחנן</t>
+  </si>
+  <si>
+    <t xml:space="preserve">יעד סיום board 06.07 · הצגת זיכרון-אור (במקום iPad) לאישור</t>
+  </si>
+  <si>
     <t xml:space="preserve">📌 הקפאת ספר</t>
   </si>
   <si>
@@ -654,7 +663,7 @@
     <t xml:space="preserve">סרט Hero</t>
   </si>
   <si>
-    <t xml:space="preserve">P1–P10 ✅ (דריפט נפתר) · נותר: composite, סטילס חסרים, P12, HD, מוזיקה</t>
+    <t xml:space="preserve">P1–P10 ✅ · composite+שוט13 עד 6.7 · HD+מוזיקה אחרי 7.7</t>
   </si>
   <si>
     <t xml:space="preserve">תערוכה / לוגיסטיקה</t>
@@ -1214,7 +1223,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -2382,14 +2391,14 @@
         <v>102</v>
       </c>
       <c r="D50" s="11" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
       <c r="E50" s="11" t="n">
-        <v>46211</v>
+        <v>46208</v>
       </c>
       <c r="F50" s="8" t="n">
         <f aca="false">E50-D50+1</f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G50" s="12" t="s">
         <v>18</v>
@@ -2412,11 +2421,11 @@
         <v>46206</v>
       </c>
       <c r="E51" s="16" t="n">
-        <v>46209</v>
+        <v>46206</v>
       </c>
       <c r="F51" s="13" t="n">
         <f aca="false">E51-D51+1</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G51" s="17" t="s">
         <v>25</v>
@@ -2436,17 +2445,17 @@
         <v>108</v>
       </c>
       <c r="D52" s="11" t="n">
-        <v>46211</v>
+        <v>46207</v>
       </c>
       <c r="E52" s="11" t="n">
-        <v>46219</v>
+        <v>46209</v>
       </c>
       <c r="F52" s="8" t="n">
         <f aca="false">E52-D52+1</f>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="H52" s="10" t="s">
         <v>109</v>
@@ -2463,14 +2472,14 @@
         <v>111</v>
       </c>
       <c r="D53" s="16" t="n">
-        <v>46209</v>
+        <v>46211</v>
       </c>
       <c r="E53" s="16" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="F53" s="13" t="n">
         <f aca="false">E53-D53+1</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G53" s="17" t="s">
         <v>53</v>
@@ -2490,14 +2499,14 @@
         <v>114</v>
       </c>
       <c r="D54" s="11" t="n">
-        <v>46213</v>
+        <v>46210</v>
       </c>
       <c r="E54" s="11" t="n">
-        <v>46223</v>
+        <v>46210</v>
       </c>
       <c r="F54" s="8" t="n">
         <f aca="false">E54-D54+1</f>
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G54" s="12" t="s">
         <v>18</v>
@@ -2700,9 +2709,16 @@
       <c r="C63" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D63" s="16"/>
-      <c r="E63" s="16"/>
-      <c r="F63" s="13"/>
+      <c r="D63" s="16" t="n">
+        <v>46210</v>
+      </c>
+      <c r="E63" s="16" t="n">
+        <v>46210</v>
+      </c>
+      <c r="F63" s="13" t="n">
+        <f aca="false">E63-D63+1</f>
+        <v>1</v>
+      </c>
       <c r="G63" s="17" t="s">
         <v>25</v>
       </c>
@@ -3019,20 +3035,20 @@
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="8" t="n">
-        <v>55</v>
+      <c r="A78" s="8" t="s">
+        <v>158</v>
       </c>
       <c r="B78" s="9" t="s">
         <v>153</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D78" s="11" t="n">
-        <v>46229</v>
+        <v>46210</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>46229</v>
+        <v>46210</v>
       </c>
       <c r="F78" s="8" t="n">
         <f aca="false">E78-D78+1</f>
@@ -3042,58 +3058,58 @@
         <v>25</v>
       </c>
       <c r="H78" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="13" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B79" s="14" t="s">
         <v>153</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D79" s="16" t="n">
-        <v>46237</v>
+        <v>46229</v>
       </c>
       <c r="E79" s="16" t="n">
-        <v>46239</v>
+        <v>46229</v>
       </c>
       <c r="F79" s="13" t="n">
         <f aca="false">E79-D79+1</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G79" s="17" t="s">
         <v>25</v>
       </c>
       <c r="H79" s="15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="8" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B80" s="9" t="s">
         <v>153</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D80" s="11" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="F80" s="8" t="n">
         <f aca="false">E80-D80+1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G80" s="12" t="s">
-        <v>163</v>
+        <v>25</v>
       </c>
       <c r="H80" s="10" t="s">
         <v>164</v>
@@ -3101,7 +3117,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="13" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B81" s="14" t="s">
         <v>153</v>
@@ -3110,10 +3126,10 @@
         <v>165</v>
       </c>
       <c r="D81" s="16" t="n">
-        <v>46240</v>
+        <v>46238</v>
       </c>
       <c r="E81" s="16" t="n">
-        <v>46240</v>
+        <v>46238</v>
       </c>
       <c r="F81" s="13" t="n">
         <f aca="false">E81-D81+1</f>
@@ -3122,7 +3138,34 @@
       <c r="G81" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="H81" s="15"/>
+      <c r="H81" s="15" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="B82" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C82" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="D82" s="11" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E82" s="11" t="n">
+        <v>46240</v>
+      </c>
+      <c r="F82" s="8" t="n">
+        <f aca="false">E82-D82+1</f>
+        <v>1</v>
+      </c>
+      <c r="G82" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="H82" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -3169,7 +3212,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -3179,22 +3222,22 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3217,7 +3260,7 @@
         <v>103</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3240,7 +3283,7 @@
         <v>64</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3248,7 +3291,7 @@
         <v>64</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C5" s="21" t="n">
         <f aca="false">MIN('Project Plan'!D31:D46)</f>
@@ -3263,7 +3306,7 @@
         <v>95</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3271,7 +3314,7 @@
         <v>98</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C6" s="21" t="n">
         <f aca="false">MIN('Project Plan'!D49:D54)</f>
@@ -3279,14 +3322,14 @@
       </c>
       <c r="D6" s="21" t="n">
         <f aca="false">MAX('Project Plan'!E49:E54)</f>
-        <v>46223</v>
+        <v>46213</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">D6-C6+1</f>
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3294,7 +3337,7 @@
         <v>117</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C7" s="21" t="n">
         <f aca="false">MIN('Project Plan'!D57:D71)</f>
@@ -3309,7 +3352,7 @@
         <v>67</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3317,14 +3360,14 @@
         <v>153</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C8" s="21" t="n">
-        <f aca="false">MIN('Project Plan'!D76:D81)</f>
+        <f aca="false">MIN('Project Plan'!D76:D82)</f>
         <v>46175</v>
       </c>
       <c r="D8" s="21" t="n">
-        <f aca="false">MAX('Project Plan'!E76:E81)</f>
+        <f aca="false">MAX('Project Plan'!E76:E82)</f>
         <v>46240</v>
       </c>
       <c r="E8" s="22" t="n">
@@ -3332,7 +3375,7 @@
         <v>66</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>